<commit_message>
updated on 25th august
</commit_message>
<xml_diff>
--- a/12627834.xlsx
+++ b/12627834.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4929e24890d5afa0/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4929e24890d5afa0/Desktop/CAP-776/CAP-776/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="76" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4D28C003-DE05-4AFB-9431-1628CB605960}"/>
+  <xr:revisionPtr revIDLastSave="77" documentId="8_{B77C434B-7271-4DC5-97B4-D8EF94629151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{02EC043D-67F3-41CA-B129-D9FB52E4F6E2}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -507,10 +507,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1241,7 +1237,7 @@
     </row>
     <row r="11" spans="1:14" x14ac:dyDescent="0.35">
       <c r="A11" s="13">
-        <v>46257</v>
+        <v>46258</v>
       </c>
       <c r="B11" s="14">
         <v>480</v>

</xml_diff>